<commit_message>
Updated datasets with better records. Completed progress report
</commit_message>
<xml_diff>
--- a/Code/dataset/Scrum_Meeting_Data_Bad_Communication.xlsx
+++ b/Code/dataset/Scrum_Meeting_Data_Bad_Communication.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benmi\Documents\GitHub\Thesis\Code\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{68F0800B-9D50-43C5-B4E6-4435AEEBFA02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6B62E0-E852-42B1-99E4-7F1CC0DAFE80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="1830" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2577,6 +2577,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -3651,6 +3656,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D301"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -16323,6 +16331,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>